<commit_message>
QC rules for SamplingPoint (SPO) table
https://taskman.eionet.europa.eu/issues/303815
Upload excel with last details
Added new view Airquality_R3.qc.[SPO_PK_CHECK_REFERENCE] that checks also AssessmentMethodId against reference table
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E8A8C4-1286-47EA-B4CF-DD5483BA8564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16EEDFF1-5A31-4F3B-AF9B-780B76EE1222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="136">
   <si>
     <t>Table</t>
   </si>
@@ -353,9 +353,6 @@
   </si>
   <si>
     <t>no modifications</t>
-  </si>
-  <si>
-    <t>Changed fiels names</t>
   </si>
   <si>
     <t>airqualitynetwork</t>
@@ -467,12 +464,44 @@
       <t xml:space="preserve"> from comparing pollutantID  to  ID, not notation(a suffix of ID field after aq/pollutant/)</t>
     </r>
   </si>
+  <si>
+    <t> SamplingPointLocation (SPL) table</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Changed field names . </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Removed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: --AirQualityStationArea,	--AirQualitySPOType, 	--SuperSite, 	--Latitude,   -- Longitude,	--[Altitude(masl)] AS Altitude_masl,	--[InletHeight(m)] AS InletHeight_m,   -- BuildingDistance(m)] AS BuildingDistance_m,   -- [KerbDistance(m)] AS KerbDistance_m</t>
+    </r>
+  </si>
+  <si>
+    <t>current view is not checkin that AssessmentMethodId exists in the reference data flow. Check  [qc].[SPO_PK_CHECK_REFERENCE]</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +525,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -530,10 +567,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -549,8 +587,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -1051,7 +1094,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1108,7 +1151,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
         <v>31</v>
@@ -1131,7 +1174,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1154,7 +1197,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
         <v>35</v>
@@ -1254,31 +1297,31 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" t="s">
         <v>110</v>
-      </c>
-      <c r="B15" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1286,53 +1329,53 @@
         <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s">
         <v>120</v>
       </c>
-      <c r="B21" t="s">
-        <v>121</v>
-      </c>
       <c r="D21" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1386,7 +1429,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1540,10 +1583,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B12" t="s">
         <v>105</v>
-      </c>
-      <c r="B12" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1551,7 +1594,7 @@
         <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1567,7 +1610,7 @@
         <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1590,7 +1633,7 @@
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="45" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="54.28515625" customWidth="1"/>
-    <col min="8" max="8" width="80.85546875" customWidth="1"/>
+    <col min="8" max="8" width="109.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1621,7 +1664,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1650,7 +1693,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1661,7 +1704,7 @@
         <v>67</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D4" t="s">
         <v>74</v>
@@ -1673,7 +1716,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1696,10 +1739,10 @@
         <v>1</v>
       </c>
       <c r="G5" s="3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -1712,14 +1755,14 @@
       <c r="D6" t="s">
         <v>78</v>
       </c>
-      <c r="E6" t="s">
-        <v>104</v>
+      <c r="E6" s="7" t="s">
+        <v>134</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1736,13 +1779,16 @@
         <v>79</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G7" s="3" t="b">
         <v>0</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1759,13 +1805,16 @@
         <v>80</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>0</v>
       </c>
       <c r="G8" s="3" t="b">
         <v>0</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1778,17 +1827,20 @@
       <c r="C9" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="8" t="s">
         <v>101</v>
       </c>
       <c r="E9" t="s">
         <v>103</v>
       </c>
       <c r="F9" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1865,10 +1917,13 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D9" r:id="rId1" xr:uid="{8434D523-4B61-4D7E-B224-82142D043008}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
QC rules for MeasurementStation (STA) table
https://taskman.eionet.europa.eu/issues/303813
[qc].[STA_03_A] changed StationNationalCode --> StationEoICode.
Added condition for CHECKING network is ALPHANUMERIC AND MIN LENGTH = 3 (or this condition is only checked in [qc].[STA_07_A]?? COMMENTED
[qc].[STA_07_A]changed StationNationalCode --> StationEoICode.
[qc].[STA_0]changed StationNationalCode --> StationEoICode.
[qc].[STA_PK]changed StationNationalCode --> StationEoICode.
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16EEDFF1-5A31-4F3B-AF9B-780B76EE1222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6016578E-5B1E-4503-B737-7BBCA39E29AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
+    <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="136">
   <si>
     <t>Table</t>
   </si>
@@ -154,18 +154,6 @@
     <t>check if the code of measurement equipment reported in SamplingProcess table appears in the Vocabulary table in the reference data flow</t>
   </si>
   <si>
-    <t>[qc].[STA.03.A]</t>
-  </si>
-  <si>
-    <t>[qc].[STA.05.A]</t>
-  </si>
-  <si>
-    <t>[qc].[STA.06.A]</t>
-  </si>
-  <si>
-    <t>[qc].[STA.07.A]</t>
-  </si>
-  <si>
     <t>[qc].[STA_0]</t>
   </si>
   <si>
@@ -190,9 +178,6 @@
     <t>https://taskman.eionet.europa.eu/issues/290540</t>
   </si>
   <si>
-    <t>Uniqueness within the same CountryCode: each AirQualityNetwork should be uniquely defined per country. &amp; Format validation: the value should conform to the expected identifier structure for air quality networks.</t>
-  </si>
-  <si>
     <t>https://taskman.eionet.europa.eu/issues/290541</t>
   </si>
   <si>
@@ -205,9 +190,6 @@
     <t>https://taskman.eionet.europa.eu/issues/290543</t>
   </si>
   <si>
-    <t>The AirQualityStationEoICode is the official Exchange of Information (EoI) identifier for the air quality station and must be unique within each reported CountryCode.</t>
-  </si>
-  <si>
     <t>The values reported under CountryCode and AirQualityStationEoICode cannot be null and the combination must be unique in the Station table.</t>
   </si>
   <si>
@@ -223,33 +205,12 @@
     <t>Changed:Table name &amp; Changed column names: airqualitynetworkorganisationallevel --&gt; "NetworkOrganisationalLevel"</t>
   </si>
   <si>
-    <t>Changed:Table name &amp; Changed column names: "airqualitynetwork" --&gt;"networkid" ; "AirQualityStationEoICode"--&gt;StationNationalCode</t>
-  </si>
-  <si>
-    <t>airqualitystationeoicode --&gt;StationNationalCode</t>
-  </si>
-  <si>
-    <t>Changed:Table name &amp; Changed column names: AirQualityStationEoICode--&gt;StationNationalCode  ;AirQualityNetwork--&gt;NetworkId  ; AirQualityNetworkOrganisationalLevel--&gt;NetworkOrganisationalLevel</t>
-  </si>
-  <si>
-    <t>airqualitystationeoicode--&gt;StationNationalCode</t>
-  </si>
-  <si>
     <t>https://taskman.eionet.europa.eu/issues/303815</t>
   </si>
   <si>
     <t>SamplingPoint (SPO)</t>
   </si>
   <si>
-    <t>[qc].[SPO.03.A]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO.03.B]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO.04.A]</t>
-  </si>
-  <si>
     <t>[qc].[SPO_0]</t>
   </si>
   <si>
@@ -359,9 +320,6 @@
   </si>
   <si>
     <t>networkid</t>
-  </si>
-  <si>
-    <t>StationNationalCode</t>
   </si>
   <si>
     <t>NetworkOrganisationalLevel</t>
@@ -496,12 +454,75 @@
   <si>
     <t>current view is not checkin that AssessmentMethodId exists in the reference data flow. Check  [qc].[SPO_PK_CHECK_REFERENCE]</t>
   </si>
+  <si>
+    <t>[qc].[STA_03_A]</t>
+  </si>
+  <si>
+    <t>[qc].[STA_05_A]</t>
+  </si>
+  <si>
+    <t>[qc].[STA_06_A]</t>
+  </si>
+  <si>
+    <t>[qc].[STA_07_A]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_03_A]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_03_B]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_04_A]</t>
+  </si>
+  <si>
+    <t>The combination of values reported under CountryCode, AirQualityStationEoICode and AirQualityNetwork must be unique in the Station table. &amp; Format validation: the value should conform to the expected identifier structure for air quality networks.</t>
+  </si>
+  <si>
+    <t>The AirQualityStationEoICode is the official Exchange of Information (EoI) identifier for the air quality station and must follow the official format used for EoI identification: &lt;CountryCode&gt;&lt;AlphanumericStationID&gt; Example: AD0942A</t>
+  </si>
+  <si>
+    <t>airqualitystationeoicode --&gt;StationEoICode</t>
+  </si>
+  <si>
+    <t>Changed:Table name &amp; Changed column names: "airqualitynetwork" --&gt;"networkid" ; "AirQualityStationEoICode"--&gt;StationEoICode</t>
+  </si>
+  <si>
+    <t>Changed:Table name &amp; Changed column names: AirQualityStationEoICode--&gt;StationEoICode  ;AirQualityNetwork--&gt;NetworkId  ; AirQualityNetworkOrganisationalLevel--&gt;NetworkOrganisationalLevel</t>
+  </si>
+  <si>
+    <t>airqualitystationeoicode--&gt;StationEoICode</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Until a formal pattern or code list is published, only uniqueness and basic format structure. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">PATTERN DEFINED in STA_07_A  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>. DOUBT: should it be strict alphanumeric, or strings are also allowed? Is this checked in STA_07_A? Commented code in [STA_03_A]:  CHECKING ALPHANUMERIC AND MIN LENGTH = 3</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -537,6 +558,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -571,7 +605,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -591,6 +625,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -663,7 +698,7 @@
     <tableColumn id="3" xr3:uid="{56291FA4-385C-46FF-8F70-79604441008F}" name="Task"/>
     <tableColumn id="4" xr3:uid="{128D8151-FD11-4D56-8FB5-B02376468273}" name="Status"/>
     <tableColumn id="5" xr3:uid="{D84F544C-7F1C-46C0-9BAF-0EC6D1B7ABA6}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{13285786-C243-403F-8480-53BBF725F280}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -691,7 +726,7 @@
     <tableColumn id="3" xr3:uid="{AC7E9942-5702-45C0-AFF2-962404B26E90}" name="Task"/>
     <tableColumn id="4" xr3:uid="{5CCAF6EA-F889-4B76-B975-51CEFEB102C1}" name="Status"/>
     <tableColumn id="5" xr3:uid="{8D9CB194-4568-4C0D-BA9A-26AF4132FBC4}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{1E881AC7-465E-4380-BB30-8C6CD89DE818}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1068,10 +1103,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1094,7 +1129,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1151,7 +1186,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
         <v>31</v>
@@ -1174,7 +1209,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1197,7 +1232,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
         <v>35</v>
@@ -1286,10 +1321,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1297,85 +1332,85 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="B22" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1398,15 +1433,15 @@
     <col min="4" max="4" width="44.85546875" customWidth="1"/>
     <col min="5" max="5" width="61" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="71.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="185.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1429,7 +1464,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1437,188 +1472,192 @@
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>122</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>132</v>
       </c>
       <c r="F3" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>123</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>124</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" t="s">
         <v>52</v>
       </c>
-      <c r="D5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" t="s">
-        <v>58</v>
-      </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G5" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>131</v>
       </c>
       <c r="F6" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="F7" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>134</v>
       </c>
       <c r="F8" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1638,10 +1677,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1664,7 +1703,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1672,19 +1711,19 @@
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -1693,24 +1732,24 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="D4" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
@@ -1721,19 +1760,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -1744,19 +1783,19 @@
     </row>
     <row r="6" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -1767,19 +1806,19 @@
     </row>
     <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>0</v>
@@ -1788,24 +1827,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>0</v>
@@ -1814,24 +1853,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
@@ -1840,79 +1879,79 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QC rules for SamplingPointLocation (SPL) table
https://taskman.eionet.europa.eu/issues/304489
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A59BB6-1483-4ADD-9CCE-A8EB0468DBDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBFFD7C-3026-41D2-A4CA-F2271BC2528D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
+    <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
     <sheet name="MeasurementStation (STA)" sheetId="2" r:id="rId2"/>
     <sheet name="SamplingPoint (SPO)" sheetId="3" r:id="rId3"/>
+    <sheet name="SamplingPointLocation (SPL) " sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="144">
   <si>
     <t>Table</t>
   </si>
@@ -452,9 +453,6 @@
     </r>
   </si>
   <si>
-    <t>current view is not checkin that AssessmentMethodId exists in the reference data flow. Check  [qc].[SPO_PK_CHECK_REFERENCE]</t>
-  </si>
-  <si>
     <t>[qc].[STA_03_A]</t>
   </si>
   <si>
@@ -516,6 +514,33 @@
       </rPr>
       <t>. DOUBT: should it be strict alphanumeric, or strings are also allowed? Is this checked in STA_07_A? Commented code in [STA_03_A]:  CHECKING ALPHANUMERIC AND MIN LENGTH = 3</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SamplingPointLocation (SPL) </t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/304489</t>
+  </si>
+  <si>
+    <t> SamplingPointLocation (SPL)  NEW table</t>
+  </si>
+  <si>
+    <t>changed rule code and table</t>
+  </si>
+  <si>
+    <t>current view is not checkin that AssessmentMethodId exists in the reference data flow. Check  [qc].[SPO_PK_CHECK_REFERENCE_TEST]</t>
+  </si>
+  <si>
+    <t>[qc].[SPL_05_A]</t>
+  </si>
+  <si>
+    <t>[qc].[SPL_05_B]</t>
+  </si>
+  <si>
+    <t>AirQualityStationArea </t>
+  </si>
+  <si>
+    <t>StationArea</t>
   </si>
 </sst>
 </file>
@@ -631,7 +656,14 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -698,7 +730,7 @@
     <tableColumn id="3" xr3:uid="{56291FA4-385C-46FF-8F70-79604441008F}" name="Task"/>
     <tableColumn id="4" xr3:uid="{128D8151-FD11-4D56-8FB5-B02376468273}" name="Status"/>
     <tableColumn id="5" xr3:uid="{D84F544C-7F1C-46C0-9BAF-0EC6D1B7ABA6}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{13285786-C243-403F-8480-53BBF725F280}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -726,7 +758,7 @@
     <tableColumn id="3" xr3:uid="{AC7E9942-5702-45C0-AFF2-962404B26E90}" name="Task"/>
     <tableColumn id="4" xr3:uid="{5CCAF6EA-F889-4B76-B975-51CEFEB102C1}" name="Status"/>
     <tableColumn id="5" xr3:uid="{8D9CB194-4568-4C0D-BA9A-26AF4132FBC4}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{1E881AC7-465E-4380-BB30-8C6CD89DE818}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -754,7 +786,7 @@
     <tableColumn id="3" xr3:uid="{BC41AFC7-AB89-4EA0-8692-93F0EA0E5A62}" name="Task"/>
     <tableColumn id="4" xr3:uid="{F7F8DB86-8A2E-4B26-A37D-351769CEBF7E}" name="Status"/>
     <tableColumn id="5" xr3:uid="{0B67C761-FAC7-459A-AC1B-D7F1B17730A0}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{7C3A4366-B4E5-4CD6-A63F-76E147C66CF2}" name="Tested" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{7C3A4366-B4E5-4CD6-A63F-76E147C66CF2}" name="Tested" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{FFE9CA48-3C44-41AB-8B0A-661E22B273DF}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -769,6 +801,34 @@
     <tableColumn id="2" xr3:uid="{9561DF00-7001-4B42-AF25-22467E4FA0E4}" name="NEW name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{219463B2-F788-41C4-AABC-02180E6CFCF5}" name="Table1347" displayName="Table1347" ref="A2:H4" totalsRowShown="0">
+  <autoFilter ref="A2:H4" xr:uid="{219463B2-F788-41C4-AABC-02180E6CFCF5}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{3EA7E6CA-FBB6-4871-BBAE-DB490EE5536B}" name="Table"/>
+    <tableColumn id="2" xr3:uid="{D0A50CC0-9F77-4704-B3A1-269A1AB52C89}" name="QC rule"/>
+    <tableColumn id="7" xr3:uid="{E1D2FAE0-8791-4006-8836-F50B526522CD}" name="Description"/>
+    <tableColumn id="3" xr3:uid="{E8B52380-3BB8-4762-B0D3-E8724AC89707}" name="Task"/>
+    <tableColumn id="4" xr3:uid="{6C05499D-8548-427F-874B-088ACF2B812C}" name="Status"/>
+    <tableColumn id="5" xr3:uid="{427C96AB-C0DB-4CCA-9908-E774BCA18601}" name="Github"/>
+    <tableColumn id="8" xr3:uid="{AFB557EE-1A5A-4BFE-85B6-53FC335EA77B}" name="Tested" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{2DD4B7F9-BC5A-475B-8B21-8EAE919D1194}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}" name="Table9" displayName="Table9" ref="A8:B15" totalsRowShown="0">
+  <autoFilter ref="A8:B15" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{CA9C040E-B181-4878-A30C-5BFA7357781D}" name="OLD name"/>
+    <tableColumn id="2" xr3:uid="{71B028CA-E61C-4941-ABF2-5B3088073D8D}" name="NEW name"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1092,11 +1152,11 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
     <col min="3" max="3" width="39.140625" customWidth="1"/>
-    <col min="4" max="4" width="60.7109375" customWidth="1"/>
-    <col min="5" max="5" width="80.28515625" customWidth="1"/>
+    <col min="4" max="4" width="43.85546875" customWidth="1"/>
+    <col min="5" max="5" width="57.5703125" customWidth="1"/>
     <col min="6" max="7" width="13.42578125" customWidth="1"/>
     <col min="8" max="8" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1155,7 +1215,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1178,7 +1238,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1293,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1316,7 +1376,7 @@
         <v>1</v>
       </c>
       <c r="G10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1351,15 +1411,18 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>98</v>
       </c>
       <c r="B17" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G17">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -1367,12 +1430,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>104</v>
       </c>
@@ -1380,7 +1443,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>105</v>
       </c>
@@ -1394,7 +1457,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>108</v>
       </c>
@@ -1408,7 +1471,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>109</v>
       </c>
@@ -1475,16 +1538,16 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
         <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -1493,7 +1556,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
@@ -1501,7 +1564,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>46</v>
@@ -1524,7 +1587,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>47</v>
@@ -1547,16 +1610,16 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D6" t="s">
         <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -1579,7 +1642,7 @@
         <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
@@ -1602,7 +1665,7 @@
         <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>1</v>
@@ -1714,7 +1777,7 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>62</v>
@@ -1740,7 +1803,7 @@
         <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>117</v>
@@ -1763,7 +1826,7 @@
         <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
         <v>63</v>
@@ -1879,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1965,4 +2028,131 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{449D902A-65C4-498F-BA40-13C5359F9E88}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="4" width="31.5703125" customWidth="1"/>
+    <col min="5" max="5" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{BC779398-DC11-4A5B-9091-6E887EA6185F}"/>
+    <hyperlink ref="B1" r:id="rId2" xr:uid="{14AB6337-B5C4-4CCB-B24C-53A82396D507}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update AQD R3 DDBB views 2026.xlsx
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBFFD7C-3026-41D2-A4CA-F2271BC2528D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0371943A-29E1-4A04-9886-4E4C8F959513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
   </bookViews>
@@ -822,8 +822,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}" name="Table9" displayName="Table9" ref="A8:B15" totalsRowShown="0">
-  <autoFilter ref="A8:B15" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}" name="Table9" displayName="Table9" ref="A8:B9" totalsRowShown="0">
+  <autoFilter ref="A8:B9" xr:uid="{EDFF03D4-E934-4919-82F6-3A28683FEA08}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{CA9C040E-B181-4878-A30C-5BFA7357781D}" name="OLD name"/>
     <tableColumn id="2" xr3:uid="{71B028CA-E61C-4941-ABF2-5B3088073D8D}" name="NEW name"/>

</xml_diff>

<commit_message>
QC rules for SamplingProcess (SPP) table
deletion of old rules:https://taskman.eionet.europa.eu/issues/303816#note-9
addition of new rules: https://taskman.eionet.europa.eu/issues/303816#note-10
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3A3251-3CB5-48BF-88FD-7509149B2046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFC1A33-6C87-4431-96DD-F97B552328E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{A21B5CE2-0BD6-4BA6-B268-6CCA106B0BAA}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="212">
   <si>
     <t>Table</t>
   </si>
@@ -122,12 +122,6 @@
     <t>check if the code of measurement type reported in SamplingProcess table appears in the Vocabulary table in the reference data flow</t>
   </si>
   <si>
-    <t>Corrected column names: "samplingmethod" --&gt; method</t>
-  </si>
-  <si>
-    <t>Corrected column names: "samplingequipment"--&gt; equipment</t>
-  </si>
-  <si>
     <t>Corrected column names</t>
   </si>
   <si>
@@ -344,12 +338,6 @@
     <t xml:space="preserve">[qc].[SPP_10_A] </t>
   </si>
   <si>
-    <t>WHERE  vocabulary = 'measurementmethod' / WHERE vocabulary = 'samplingmethod'</t>
-  </si>
-  <si>
-    <t>WHERE vocabulary = 'measurementequipment' / WHERE vocabulary = 'samplingequipment'</t>
-  </si>
-  <si>
     <t>PollutantID</t>
   </si>
   <si>
@@ -372,15 +360,6 @@
   </si>
   <si>
     <t>ProcessDocumentationId</t>
-  </si>
-  <si>
-    <t>Conflict between[qc].[SPP_10_A] and [qc].[SPP_08_A]</t>
-  </si>
-  <si>
-    <t>New vocabulary table in process</t>
-  </si>
-  <si>
-    <t>Conflict between[qc].[SPP_09_A] and [qc].[SPP_11_A]</t>
   </si>
   <si>
     <t>[qc].[SPP_08_A]</t>
@@ -543,9 +522,6 @@
     <t>STA_07 is StationNationalCode and it is of less importance, although we may have some basic check testing the length perhaps, it is varchar(50), STA_07_A?</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
-  </si>
-  <si>
     <t>STA_03_B</t>
   </si>
   <si>
@@ -589,9 +565,6 @@
     <t xml:space="preserve"> STA_01_A</t>
   </si>
   <si>
-    <t>country code can be checked against vocabulary?</t>
-  </si>
-  <si>
     <t>PROPOSED CHANGES DOUBTS</t>
   </si>
   <si>
@@ -631,7 +604,237 @@
     <t xml:space="preserve"> testing the length NetworkId ? What lenght shoul it be?50?</t>
   </si>
   <si>
-    <t>current view is not checkin that AssessmentMethodId exists in the reference THIS IS OK</t>
+    <r>
+      <t xml:space="preserve">current view is not checkin that AssessmentMethodId exists in the reference </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>THIS IS OK</t>
+    </r>
+  </si>
+  <si>
+    <t>DELETED</t>
+  </si>
+  <si>
+    <t>SPP_01_A</t>
+  </si>
+  <si>
+    <t>SPP_02_A</t>
+  </si>
+  <si>
+    <t>SPP_03_A</t>
+  </si>
+  <si>
+    <t>SPP_03_B</t>
+  </si>
+  <si>
+    <t>SPP_04_B</t>
+  </si>
+  <si>
+    <t>SPP_04_A</t>
+  </si>
+  <si>
+    <t>SPP_04_C</t>
+  </si>
+  <si>
+    <t>SPP_05_A</t>
+  </si>
+  <si>
+    <t>SPP_06_A</t>
+  </si>
+  <si>
+    <t>SPP_06_B</t>
+  </si>
+  <si>
+    <t>SPP_07_B</t>
+  </si>
+  <si>
+    <t>SPP_14_A</t>
+  </si>
+  <si>
+    <t>SPP_12_A</t>
+  </si>
+  <si>
+    <t>SPP_13_A</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_01 must correspond to one of the values of Notation in [Airquality_R3].[reference].[Vocabulary] where vocabulary = 'countries'.QC name: SPP_01_A Vocabulary – [CountryCode]</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_02 must have length &gt; 0 and &lt; 151.QC name: SPP_02_A Constraint – [ProcessId]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QC rule description: Attribute SPP_03 must correspond to one of the values of attribute AssessmentMethodId (SPO_02) for the same CountryCode (SPO_01) in SamplingPoint table in reporting or reference data. QC name: SPP_03_B Consistency &amp; Cross-check – [CountryCode] SPO_01 [AssessmentMethodId] SPO_02 </t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_04 value must be &lt;= SPP_05 if SPP_05 is not null (when SPP_04 = SPP_05 the record is meant for deletion) QC name: SPP_04_A Consistency  – [ProcessActivityEnd] SPP_05</t>
+  </si>
+  <si>
+    <t>QC rule description: For every new [ProcessActivityBegin] within the same CountryCode and AssessmentMethodId, all other [ProcessActivityBegin] must be accompanied by [ProcessActivityEnd] &amp; the new [ProcessActivityBegin] must be &gt;= latest [ProcessActivityEnd]  QC name: SPP_04_B Consistency – [ProcessActivityEnd] SPP_05</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_04 must follow ISO8601, e.g. '2025-01-01T00:00:00' for UTC/Zulu or '2025-01-01T00:00:00+02:00' for UTC+2. QC name: SPP_04_C Format – [ProcessActivityBegin]</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_05 must follow ISO8601, e.g. '2025-01-01T00:00:00' for UTC/Zulu or '2025-01-01T00:00:00+02:00' for UTC+2  QC name: SPP_05_A Format – [ProcessActivityEnd]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QC rule description: Attribute SPP_06 value must correspond to one of the values of cast(replace([URI],'http://dd.eionet.europa.eu/vocabulary/aq/pollutant/','') as integer) from [Airquality_R3].[reference].[Vocabulary] where vocabulary = 'pollutant'  QC name: SPP_06_A Vocabulary - [PollutantId] </t>
+  </si>
+  <si>
+    <t>QC rule description: Combination of attribute values SPP_03 and SPP_06 must correspond to the combination of attribute values SPO_02 and SPO_04 in SamplingPoint table in reporting or reference data.QC name: SPP_06_B Cross-check &amp; Consistency - [AssessmentMethodId] SPO_02 [PollutantId] SPO_04</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_07 must have length &gt; 0 and &lt; 51. QC name: SPP_07_B Constraint – [MeasurementType length]</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_12 must correspond to one of the values of attribute DocumentId (DOC_04) in Documentation table in reporting or reference data. QC name: SPP_12_A Cross-check - [DocumentId] DOC_04</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_13 must correspond to one of the values of attribute DocumentId (DOC_04) in Documentation table in reporting or reference data. QC name: SPP_13_A Cross-check - [DocumentId] DOC_04</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_14 must correspond to one of the values of attribute DocumentId (DOC_04) in Documentation table in reporting or reference data. QC name: SPP_14_A Cross-check - [DocumentId] DOC_04</t>
+  </si>
+  <si>
+    <t>country code can be checked against vocabulary ' Countries'</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303813#note-10</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303813#note-11</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303813#note-12</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-10</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-11</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-12</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-13</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-14</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-15</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-16</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-17</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-18</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-19</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-20</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-21</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-22</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/303816#note-23</t>
+  </si>
+  <si>
+    <t>STA_01_A Vocabulary - [CountryCode]</t>
+  </si>
+  <si>
+    <t>QC rule description: Attribute SPP_03 must have length &gt; 0 and &lt; 51.. QC name: SPP_03_A Constraint – [AssessmentMethodId]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should we select too the records where both dates are equal? </t>
+  </si>
+  <si>
+    <t>CREATE OR ALTER VIEW [qc].[SPP_04_B] AS
+WITH src AS (
+SELECT
+[CountryCode],
+[AssessmentMethodId],
+[ProcessActivityBegin],
+[ProcessActivityEnd],
+-- Robust parsing (keeps NULL if empty/invalid)
+TRY_CONVERT(datetimeoffset(0),
+NULLIF(LTRIM(RTRIM(CONVERT(nvarchar(50), [ProcessActivityBegin]))), ''),
+126) AS Begin_dt,
+TRY_CONVERT(datetimeoffset(0),
+NULLIF(LTRIM(RTRIM(CONVERT(nvarchar(50), [ProcessActivityEnd]))), ''),
+126) AS End_dt
+FROM [reporting].[SamplingProcess]
+),
+ordered AS (
+SELECT
+s.*,
+-- Latest previous End within the same (CountryCode, AssessmentMethodId)
+MAX(End_dt) OVER (
+PARTITION BY [CountryCode], [AssessmentMethodId]
+ORDER BY Begin_dt
+ROWS BETWEEN UNBOUNDED PRECEDING AND 1 PRECEDING
+) AS prev_max_end,
+-- Count of previous rows that are still open (End_dt IS NULL)
+SUM(CASE WHEN End_dt IS NULL THEN 1 ELSE 0 END) OVER (
+PARTITION BY [CountryCode], [AssessmentMethodId]
+ORDER BY Begin_dt
+ROWS BETWEEN UNBOUNDED PRECEDING AND 1 PRECEDING
+) AS prev_open_cnt
+FROM src s
+),
+violations AS (
+SELECT
+[CountryCode],
+[AssessmentMethodId],
+[ProcessActivityBegin],
+[ProcessActivityEnd],
+Begin_dt,
+End_dt,
+prev_max_end,
+CASE
+WHEN Begin_dt IS NULL
+THEN 'Begin is NULL or invalid'
+WHEN prev_open_cnt &gt; 0
+THEN 'Previous interval without End exists'
+WHEN prev_max_end IS NOT NULL AND Begin_dt &lt; prev_max_end
+THEN 'Begin earlier than latest previous End'
+END AS violation
+FROM ordered
+WHERE
+Begin_dt IS NULL
+OR prev_open_cnt &gt; 0
+OR (prev_max_end IS NOT NULL AND Begin_dt &lt; prev_max_end)
+)
+SELECT
+[CountryCode],
+[AssessmentMethodId],
+[ProcessActivityBegin],
+[ProcessActivityEnd],
+violation,
+prev_max_end AS [LatestPreviousEnd]
+FROM violations;
+GO</t>
+  </si>
+  <si>
+    <t>Probar bien</t>
   </si>
 </sst>
 </file>
@@ -694,7 +897,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -709,8 +912,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
     <fill>
@@ -731,13 +934,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -760,7 +980,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -774,25 +994,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1">
@@ -803,18 +1020,112 @@
       </extLst>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="13">
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <extLst>
@@ -880,8 +1191,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{423CFA4E-A9B9-4105-8206-0DFCD6FBDA50}" name="Table1" displayName="Table1" ref="A2:H10" totalsRowShown="0">
-  <autoFilter ref="A2:H10" xr:uid="{423CFA4E-A9B9-4105-8206-0DFCD6FBDA50}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{423CFA4E-A9B9-4105-8206-0DFCD6FBDA50}" name="Table1" displayName="Table1" ref="A2:H24" totalsRowShown="0">
+  <autoFilter ref="A2:H24" xr:uid="{423CFA4E-A9B9-4105-8206-0DFCD6FBDA50}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{1696B22E-BC08-44CF-B50B-FDE762F9ECC6}" name="Table"/>
     <tableColumn id="2" xr3:uid="{E4B9E223-A638-4A3B-B3C4-795A9ED72AB5}" name="QC rule"/>
@@ -889,7 +1200,7 @@
     <tableColumn id="3" xr3:uid="{56291FA4-385C-46FF-8F70-79604441008F}" name="Task"/>
     <tableColumn id="4" xr3:uid="{128D8151-FD11-4D56-8FB5-B02376468273}" name="Status"/>
     <tableColumn id="5" xr3:uid="{D84F544C-7F1C-46C0-9BAF-0EC6D1B7ABA6}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{AB8475BE-CBFA-48D9-894C-C12EF21A3A72}" name="Tested" dataDxfId="11"/>
     <tableColumn id="6" xr3:uid="{13285786-C243-403F-8480-53BBF725F280}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -897,8 +1208,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6DF5A80-7E3C-4971-A9BE-A7226F720E3B}" name="Table469" displayName="Table469" ref="A13:B23" totalsRowShown="0">
-  <autoFilter ref="A13:B23" xr:uid="{A6DF5A80-7E3C-4971-A9BE-A7226F720E3B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6DF5A80-7E3C-4971-A9BE-A7226F720E3B}" name="Table469" displayName="Table469" ref="A26:B36" totalsRowShown="0">
+  <autoFilter ref="A26:B36" xr:uid="{A6DF5A80-7E3C-4971-A9BE-A7226F720E3B}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{FA2A20B4-3C91-4EB0-8FC1-5902337F208E}" name="OLD name"/>
     <tableColumn id="2" xr3:uid="{ED906FF7-EC0A-4F59-8767-758A2F568440}" name="NEW name"/>
@@ -908,8 +1219,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C3B84D44-9C67-4833-B196-916A04CB6055}" name="Table13" displayName="Table13" ref="A2:H12" totalsRowShown="0">
-  <autoFilter ref="A2:H12" xr:uid="{C3B84D44-9C67-4833-B196-916A04CB6055}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C3B84D44-9C67-4833-B196-916A04CB6055}" name="Table13" displayName="Table13" ref="A2:H13" totalsRowShown="0">
+  <autoFilter ref="A2:H13" xr:uid="{C3B84D44-9C67-4833-B196-916A04CB6055}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{0594A6FA-E910-4D63-A8AF-60D58DFC7886}" name="Table"/>
     <tableColumn id="2" xr3:uid="{674EE5E3-898C-40FC-8B1E-16E1B729A0E0}" name="QC rule"/>
@@ -917,7 +1228,7 @@
     <tableColumn id="3" xr3:uid="{AC7E9942-5702-45C0-AFF2-962404B26E90}" name="Task"/>
     <tableColumn id="4" xr3:uid="{5CCAF6EA-F889-4B76-B975-51CEFEB102C1}" name="Status"/>
     <tableColumn id="5" xr3:uid="{8D9CB194-4568-4C0D-BA9A-26AF4132FBC4}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{4FF331A0-ACA2-4685-B2F6-369D784F3BA1}" name="Tested" dataDxfId="10"/>
     <tableColumn id="6" xr3:uid="{1E881AC7-465E-4380-BB30-8C6CD89DE818}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -936,17 +1247,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{65FD295E-14D8-4D52-B1C9-A4AA3E9D9358}" name="Table1311" displayName="Table1311" ref="A22:H27" totalsRowShown="0">
-  <autoFilter ref="A22:H27" xr:uid="{65FD295E-14D8-4D52-B1C9-A4AA3E9D9358}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{65FD295E-14D8-4D52-B1C9-A4AA3E9D9358}" name="Table1311" displayName="Table1311" ref="A22:H26" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A22:H26" xr:uid="{65FD295E-14D8-4D52-B1C9-A4AA3E9D9358}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{192BAF8F-FD98-42BB-9C26-E2FE8E103ADA}" name="Table"/>
-    <tableColumn id="2" xr3:uid="{2BD013E8-570F-4856-BFB9-03670630CFC5}" name="QC rule"/>
-    <tableColumn id="7" xr3:uid="{377BEE01-1775-49C3-A18E-E09E77C299CD}" name="Description"/>
-    <tableColumn id="3" xr3:uid="{74F320D0-0AD9-4AC0-AF0E-2E2F6B3B420D}" name="Task"/>
-    <tableColumn id="4" xr3:uid="{3DB0E456-1505-4E17-9AC0-90B3B70BA5CA}" name="Status"/>
-    <tableColumn id="5" xr3:uid="{BCADBE24-4A8E-4D68-8A04-42BAF3C5FA4E}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{D2750DEC-703A-4031-9E65-CC79101CA95B}" name="Tested" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{6CF0ADAE-3BB9-49FB-9CB0-30C3A3A0468B}" name="Comments"/>
+    <tableColumn id="1" xr3:uid="{192BAF8F-FD98-42BB-9C26-E2FE8E103ADA}" name="Table" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{2BD013E8-570F-4856-BFB9-03670630CFC5}" name="QC rule" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{377BEE01-1775-49C3-A18E-E09E77C299CD}" name="Description" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{74F320D0-0AD9-4AC0-AF0E-2E2F6B3B420D}" name="Task" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{3DB0E456-1505-4E17-9AC0-90B3B70BA5CA}" name="Status" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{BCADBE24-4A8E-4D68-8A04-42BAF3C5FA4E}" name="Github" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{D2750DEC-703A-4031-9E65-CC79101CA95B}" name="Tested" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{6CF0ADAE-3BB9-49FB-9CB0-30C3A3A0468B}" name="Comments" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -962,7 +1273,7 @@
     <tableColumn id="3" xr3:uid="{BC41AFC7-AB89-4EA0-8692-93F0EA0E5A62}" name="Task"/>
     <tableColumn id="4" xr3:uid="{F7F8DB86-8A2E-4B26-A37D-351769CEBF7E}" name="Status"/>
     <tableColumn id="5" xr3:uid="{0B67C761-FAC7-459A-AC1B-D7F1B17730A0}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{7C3A4366-B4E5-4CD6-A63F-76E147C66CF2}" name="Tested" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{7C3A4366-B4E5-4CD6-A63F-76E147C66CF2}" name="Tested" dataDxfId="9"/>
     <tableColumn id="6" xr3:uid="{FFE9CA48-3C44-41AB-8B0A-661E22B273DF}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -990,7 +1301,7 @@
     <tableColumn id="3" xr3:uid="{E8B52380-3BB8-4762-B0D3-E8724AC89707}" name="Task"/>
     <tableColumn id="4" xr3:uid="{6C05499D-8548-427F-874B-088ACF2B812C}" name="Status"/>
     <tableColumn id="5" xr3:uid="{427C96AB-C0DB-4CCA-9908-E774BCA18601}" name="Github"/>
-    <tableColumn id="8" xr3:uid="{AFB557EE-1A5A-4BFE-85B6-53FC335EA77B}" name="Tested" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{AFB557EE-1A5A-4BFE-85B6-53FC335EA77B}" name="Tested" dataDxfId="12"/>
     <tableColumn id="6" xr3:uid="{2DD4B7F9-BC5A-475B-8B21-8EAE919D1194}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1325,24 +1636,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A524921F-6468-4312-9D24-8082E775F4AE}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
-    <col min="2" max="2" width="33.85546875" customWidth="1"/>
-    <col min="3" max="3" width="39.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="66.85546875" customWidth="1"/>
     <col min="4" max="4" width="43.85546875" customWidth="1"/>
-    <col min="5" max="5" width="57.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="7" width="13.42578125" customWidth="1"/>
     <col min="8" max="8" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1365,7 +1676,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1385,7 +1696,7 @@
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -1421,17 +1732,17 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>113</v>
+      <c r="B5" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -1444,17 +1755,17 @@
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>114</v>
+      <c r="B6" s="20" t="s">
+        <v>107</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -1463,49 +1774,49 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="B7" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="E7" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="F7" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="E8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3" t="b">
+      <c r="E8" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="F8" s="19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" s="19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1517,7 +1828,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -1532,15 +1843,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>32</v>
+      <c r="C10" t="s">
+        <v>30</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
@@ -1555,104 +1866,434 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" t="s">
+        <v>149</v>
+      </c>
+      <c r="F11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" t="s">
+        <v>194</v>
+      </c>
+      <c r="E12" t="s">
+        <v>149</v>
+      </c>
+      <c r="F12" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>164</v>
+      </c>
+      <c r="C13" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" t="s">
+        <v>195</v>
+      </c>
+      <c r="E13" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>94</v>
+        <v>165</v>
+      </c>
+      <c r="C14" t="s">
+        <v>178</v>
+      </c>
+      <c r="D14" t="s">
+        <v>196</v>
+      </c>
+      <c r="E14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F14" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>167</v>
+      </c>
+      <c r="C15" t="s">
+        <v>179</v>
+      </c>
+      <c r="D15" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" t="s">
+        <v>149</v>
+      </c>
+      <c r="F15" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>166</v>
+      </c>
+      <c r="C16" t="s">
+        <v>180</v>
+      </c>
+      <c r="D16" t="s">
+        <v>198</v>
+      </c>
+      <c r="E16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F16" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
-      </c>
-      <c r="G17">
-        <v>99</v>
+        <v>168</v>
+      </c>
+      <c r="C17" t="s">
+        <v>181</v>
+      </c>
+      <c r="D17" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" t="s">
+        <v>149</v>
+      </c>
+      <c r="F17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>102</v>
+        <v>169</v>
+      </c>
+      <c r="C18" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" t="s">
+        <v>200</v>
+      </c>
+      <c r="E18" t="s">
+        <v>149</v>
+      </c>
+      <c r="F18" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>170</v>
+      </c>
+      <c r="C19" t="s">
+        <v>183</v>
+      </c>
+      <c r="D19" t="s">
+        <v>201</v>
+      </c>
+      <c r="E19" t="s">
+        <v>149</v>
+      </c>
+      <c r="F19" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>111</v>
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C20" t="s">
+        <v>184</v>
+      </c>
+      <c r="D20" t="s">
+        <v>202</v>
+      </c>
+      <c r="E20" t="s">
+        <v>149</v>
+      </c>
+      <c r="F20" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>100</v>
+        <v>172</v>
+      </c>
+      <c r="C21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D21" t="s">
+        <v>203</v>
+      </c>
+      <c r="E21" t="s">
+        <v>149</v>
+      </c>
+      <c r="F21" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>101</v>
+        <v>174</v>
+      </c>
+      <c r="C22" t="s">
+        <v>186</v>
+      </c>
+      <c r="D22" t="s">
+        <v>204</v>
+      </c>
+      <c r="E22" t="s">
+        <v>149</v>
+      </c>
+      <c r="F22" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>109</v>
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23" t="s">
+        <v>205</v>
+      </c>
+      <c r="E23" t="s">
+        <v>149</v>
+      </c>
+      <c r="F23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>173</v>
+      </c>
+      <c r="C24" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" t="s">
+        <v>206</v>
+      </c>
+      <c r="E24" t="s">
+        <v>149</v>
+      </c>
+      <c r="F24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>93</v>
+      </c>
+      <c r="B28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>96</v>
+      </c>
+      <c r="B30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>100</v>
+      </c>
+      <c r="D33" s="21"/>
+      <c r="E33" s="20"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="9"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B39" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="B42" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
     <tablePart r:id="rId1"/>
@@ -1663,12 +2304,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE99D520-B7FC-4923-A065-1738A7852047}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" customWidth="1"/>
     <col min="2" max="2" width="24.140625" customWidth="1"/>
-    <col min="3" max="3" width="45.28515625" customWidth="1"/>
+    <col min="3" max="3" width="51.28515625" customWidth="1"/>
     <col min="4" max="4" width="44.85546875" customWidth="1"/>
     <col min="5" max="5" width="36.28515625" customWidth="1"/>
     <col min="6" max="7" width="13.42578125" customWidth="1"/>
@@ -1677,10 +2318,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1703,7 +2344,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -1711,19 +2352,19 @@
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -1731,25 +2372,25 @@
       <c r="G3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>134</v>
+      <c r="H3" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
@@ -1760,19 +2401,19 @@
     </row>
     <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>123</v>
+        <v>37</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>116</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>151</v>
+        <v>142</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>143</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -1781,44 +2422,44 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="16" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="18" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="18" t="b">
+    <row r="6" spans="1:8" s="13" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="15" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
@@ -1829,19 +2470,19 @@
     </row>
     <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>1</v>
@@ -1852,19 +2493,19 @@
     </row>
     <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
@@ -1875,20 +2516,20 @@
     </row>
     <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="D10" t="s">
-        <v>151</v>
-      </c>
-      <c r="E10" s="19" t="s">
         <v>158</v>
       </c>
+      <c r="D10" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>149</v>
+      </c>
       <c r="F10" s="3" t="b">
         <v>1</v>
       </c>
@@ -1896,21 +2537,24 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>158</v>
+        <v>156</v>
+      </c>
+      <c r="D11" t="s">
+        <v>190</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>149</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>1</v>
@@ -1919,21 +2563,24 @@
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>158</v>
+        <v>157</v>
+      </c>
+      <c r="D12" t="s">
+        <v>191</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>149</v>
       </c>
       <c r="F12" s="3" t="b">
         <v>1</v>
@@ -1942,53 +2589,80 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>164</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>156</v>
-      </c>
+      <c r="A21" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="B21" s="12"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -2010,107 +2684,102 @@
         <v>5</v>
       </c>
       <c r="G22" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H22" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="13" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H23"/>
+    <row r="23" spans="1:8" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A23" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" s="20"/>
     </row>
     <row r="24" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="F24" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3" t="b">
-        <v>0</v>
-      </c>
+      <c r="A24" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" s="20"/>
+      <c r="F24" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" s="20"/>
     </row>
     <row r="25" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A25" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="F25" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G25" s="3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="13" t="s">
+      <c r="A25" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G25" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" s="20"/>
+    </row>
+    <row r="26" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A26" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-    </row>
-    <row r="27" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>144</v>
-      </c>
-      <c r="B27" t="s">
-        <v>160</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F27" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G27" s="3" t="b">
-        <v>0</v>
-      </c>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" s="20"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="7"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9"/>
     </row>
     <row r="33" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
+      <c r="A33" s="9"/>
     </row>
     <row r="34" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="10"/>
@@ -2119,10 +2788,10 @@
       <c r="A35" s="11"/>
     </row>
     <row r="36" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
+      <c r="A36" s="9"/>
     </row>
     <row r="37" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="10"/>
+      <c r="A37" s="9"/>
     </row>
     <row r="38" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
@@ -2131,10 +2800,10 @@
       <c r="A39" s="11"/>
     </row>
     <row r="40" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="12"/>
+      <c r="A40" s="9"/>
     </row>
     <row r="41" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="10"/>
+      <c r="A41" s="9"/>
     </row>
     <row r="42" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10"/>
@@ -2143,28 +2812,27 @@
       <c r="A43" s="11"/>
     </row>
     <row r="44" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="12"/>
+      <c r="A44" s="9"/>
     </row>
     <row r="45" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="10"/>
+      <c r="A45" s="9"/>
     </row>
     <row r="46" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="10"/>
-    </row>
-    <row r="47" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" location="note-9" xr:uid="{72C4A5B9-C2E0-4C0D-AB8F-612F13117959}"/>
+    <hyperlink ref="D10" r:id="rId2" location="note-9" xr:uid="{11CE857E-8D11-4DD9-A7FE-0924BF76F67B}"/>
+    <hyperlink ref="D13" r:id="rId3" location="note-12" xr:uid="{E50AF0EB-E7F2-4790-90D7-2AAF09D6E2D4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
   <tableParts count="3">
-    <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2184,10 +2852,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2210,7 +2878,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -2218,19 +2886,19 @@
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -2239,24 +2907,24 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
@@ -2267,19 +2935,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -2290,19 +2958,19 @@
     </row>
     <row r="6" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>120</v>
+        <v>63</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -2313,19 +2981,19 @@
     </row>
     <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
         <v>55</v>
       </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>0</v>
@@ -2334,24 +3002,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>0</v>
@@ -2360,25 +3028,25 @@
         <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D9" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" t="s">
         <v>88</v>
       </c>
-      <c r="E9" t="s">
-        <v>90</v>
-      </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
       </c>
@@ -2386,79 +3054,79 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2488,10 +3156,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>136</v>
+        <v>39</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2514,7 +3182,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
@@ -2522,19 +3190,19 @@
     </row>
     <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" s="8" t="s">
         <v>66</v>
       </c>
+      <c r="D3" s="6" t="s">
+        <v>64</v>
+      </c>
       <c r="E3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -2543,24 +3211,24 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
@@ -2569,23 +3237,23 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>141</v>
+      <c r="A9" s="7" t="s">
+        <v>134</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New views in SPL table
Created the next views relative to SPL table:
[qc].[SPL_01_A]
[qc].[SPL_02_A]
[qc].[SPL_02_B]
[qc].[SPL_03_A]
[qc].[SPL_03_B]
[qc].[SPL_03_C]
[qc].[SPL_04_A]
[qc].[SPL_04_B]

[qc].[SPL_06_A]

[qc].[SPL_09_A]
[qc].[SPL_09_B]
[qc].[SPL_10_A]
[qc].[SPL_10_B]
[qc].[SPL_11_A]
[qc].[SPL_12_A]
[qc].[SPL_13_A]
[qc].[SPL_14_A]
[qc].[SPL_15_A]
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026.xlsx
+++ b/AQD R3 DDBB views 2026.xlsx
@@ -1013,7 +1013,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="2" applyFont="1" applyFill="1">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="2" applyFont="1" applyFill="1"/>
@@ -3118,7 +3118,8 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="28.85546875"/>
     <col customWidth="1" min="2" max="2" width="32.7109375"/>
-    <col customWidth="1" min="3" max="4" width="31.5703125"/>
+    <col customWidth="1" min="3" max="3" width="71.125"/>
+    <col customWidth="1" min="4" max="4" width="31.5703125"/>
     <col bestFit="1" customWidth="1" min="5" max="5" width="38.85546875"/>
     <col bestFit="1" min="6" max="7" width="12.0234375"/>
     <col customWidth="1" min="8" max="8" width="57.50390625"/>
@@ -3212,20 +3213,18 @@
     </row>
     <row r="5" ht="14.25">
       <c r="E5" s="19"/>
-      <c r="F5"/>
-      <c r="G5"/>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B6" t="s">
         <v>208</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="D6" s="20"/>
+      <c r="D6" s="19"/>
       <c r="E6" s="19" t="s">
         <v>210</v>
       </c>
@@ -3235,10 +3234,10 @@
       <c r="G6" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="20"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B7" t="s">
@@ -3247,7 +3246,7 @@
       <c r="C7" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="D7" s="20"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="19" t="s">
         <v>210</v>
       </c>
@@ -3257,19 +3256,19 @@
       <c r="G7" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="20"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="19" t="s">
         <v>210</v>
       </c>
@@ -3279,19 +3278,19 @@
       <c r="G8" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="20"/>
+      <c r="H8" s="19"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B9" t="s">
         <v>215</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D9" s="20"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="19" t="s">
         <v>210</v>
       </c>
@@ -3301,19 +3300,19 @@
       <c r="G9" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="20"/>
+      <c r="H9" s="19"/>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B10" t="s">
         <v>217</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="D10" s="20"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="19" t="s">
         <v>210</v>
       </c>
@@ -3323,19 +3322,19 @@
       <c r="G10" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="20"/>
+      <c r="H10" s="19"/>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B11" t="s">
         <v>219</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="D11" s="20"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="19" t="s">
         <v>210</v>
       </c>
@@ -3345,19 +3344,19 @@
       <c r="G11" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="20"/>
+      <c r="H11" s="19"/>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B12" t="s">
         <v>221</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="D12" s="20"/>
+      <c r="D12" s="19"/>
       <c r="E12" s="19" t="s">
         <v>210</v>
       </c>
@@ -3367,7 +3366,7 @@
       <c r="G12" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="20"/>
+      <c r="H12" s="19"/>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
@@ -3379,7 +3378,6 @@
       <c r="C13" t="s">
         <v>224</v>
       </c>
-      <c r="D13"/>
       <c r="E13" s="19" t="s">
         <v>210</v>
       </c>
@@ -3389,7 +3387,6 @@
       <c r="G13" t="b">
         <v>0</v>
       </c>
-      <c r="H13"/>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" t="s">
@@ -3401,7 +3398,6 @@
       <c r="C14" t="s">
         <v>225</v>
       </c>
-      <c r="D14"/>
       <c r="E14" s="19" t="s">
         <v>210</v>
       </c>
@@ -3411,10 +3407,9 @@
       <c r="G14" t="b">
         <v>0</v>
       </c>
-      <c r="H14"/>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B15" t="s">
@@ -3423,7 +3418,7 @@
       <c r="C15" t="s">
         <v>227</v>
       </c>
-      <c r="D15" s="20"/>
+      <c r="D15" s="19"/>
       <c r="E15" s="19" t="s">
         <v>210</v>
       </c>
@@ -3433,41 +3428,37 @@
       <c r="G15" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="19" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
       <c r="E16" s="19"/>
-      <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16" s="20"/>
+      <c r="H16" s="19"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="A17" s="19"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
       <c r="E17" s="19"/>
-      <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17" s="20"/>
+      <c r="H17" s="19"/>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B18" t="s">
         <v>229</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="D18" s="20"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="19" t="s">
         <v>210</v>
       </c>
@@ -3477,19 +3468,19 @@
       <c r="G18" t="b">
         <v>0</v>
       </c>
-      <c r="H18" s="20"/>
+      <c r="H18" s="19"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B19" t="s">
         <v>231</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="D19" s="20"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="19" t="s">
         <v>210</v>
       </c>
@@ -3499,19 +3490,19 @@
       <c r="G19" t="b">
         <v>0</v>
       </c>
-      <c r="H19" s="20"/>
+      <c r="H19" s="19"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B20" t="s">
         <v>233</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="D20" s="20"/>
+      <c r="D20" s="19"/>
       <c r="E20" s="19" t="s">
         <v>210</v>
       </c>
@@ -3521,19 +3512,19 @@
       <c r="G20" t="b">
         <v>0</v>
       </c>
-      <c r="H20" s="20"/>
+      <c r="H20" s="19"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B21" t="s">
         <v>235</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="D21" s="20"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="19" t="s">
         <v>210</v>
       </c>
@@ -3543,19 +3534,19 @@
       <c r="G21" t="b">
         <v>0</v>
       </c>
-      <c r="H21" s="20"/>
+      <c r="H21" s="19"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B22" t="s">
         <v>237</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="D22" s="20"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="19" t="s">
         <v>210</v>
       </c>
@@ -3565,19 +3556,19 @@
       <c r="G22" t="b">
         <v>0</v>
       </c>
-      <c r="H22" s="20"/>
+      <c r="H22" s="19"/>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B23" t="s">
         <v>239</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="D23" s="20"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="19" t="s">
         <v>210</v>
       </c>
@@ -3587,19 +3578,19 @@
       <c r="G23" t="b">
         <v>0</v>
       </c>
-      <c r="H23" s="20"/>
+      <c r="H23" s="19"/>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B24" t="s">
         <v>241</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="D24" s="20"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="19" t="s">
         <v>210</v>
       </c>
@@ -3609,19 +3600,19 @@
       <c r="G24" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="20"/>
+      <c r="H24" s="19"/>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B25" t="s">
         <v>243</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="D25" s="20"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="19" t="s">
         <v>210</v>
       </c>
@@ -3631,10 +3622,10 @@
       <c r="G25" t="b">
         <v>0</v>
       </c>
-      <c r="H25" s="20"/>
+      <c r="H25" s="19"/>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="19" t="s">
         <v>203</v>
       </c>
       <c r="B26" t="s">
@@ -3643,31 +3634,31 @@
       <c r="C26" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
     </row>
     <row r="27" ht="14.25">
-      <c r="A27" s="20"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="20"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
     </row>
     <row r="31" ht="14.25">
       <c r="A31" t="s">

</xml_diff>